<commit_message>
Update: Processed data from home
</commit_message>
<xml_diff>
--- a/根留台灣計畫/108年10-12月根留台灣委辦手續費.xlsx
+++ b/根留台灣計畫/108年10-12月根留台灣委辦手續費.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shanehsueh\Desktop\政策性貸款融資後查核\根留台灣申請委辦手續費\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eric\Downloads\KPMG\根留台灣計畫\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08C8D4E-B5B6-4767-9BB3-B3DEE808390D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="10月" sheetId="1" r:id="rId1"/>
@@ -729,21 +729,21 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:P824"/>
-  <sheetFormatPr defaultColWidth="5.375" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="5.3984375" defaultRowHeight="13.15"/>
   <cols>
     <col min="1" max="1" width="12" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.3984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.86328125" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" style="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.375" style="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="9.75" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.875" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="5.375" style="6"/>
+    <col min="8" max="8" width="10.3984375" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="9.73046875" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.3984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.86328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="5.3984375" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -761,7 +761,7 @@
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" ht="13.5">
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
@@ -773,7 +773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="18" customFormat="1" ht="27.75" thickBot="1">
+    <row r="3" spans="1:16" s="18" customFormat="1" ht="26.65" thickBot="1">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -15635,21 +15635,21 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:P826"/>
-  <sheetFormatPr defaultColWidth="5.375" defaultRowHeight="13.5" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="5.3984375" defaultRowHeight="13.15" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="16" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.3984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.86328125" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1328125" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" style="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.375" style="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="9.75" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.125" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="5.375" style="6"/>
+    <col min="8" max="8" width="10.3984375" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="9.73046875" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.3984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="5.3984375" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -15667,7 +15667,7 @@
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" ht="13.5">
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
@@ -15679,7 +15679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="18" customFormat="1" ht="27.75" thickBot="1">
+    <row r="3" spans="1:16" s="18" customFormat="1" ht="26.65" thickBot="1">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -15763,7 +15763,7 @@
         <v>38000000</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="18" customFormat="1" outlineLevel="1">
+    <row r="5" spans="1:16" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A5" s="25" t="s">
         <v>28</v>
       </c>
@@ -15832,7 +15832,7 @@
         <v>190000000</v>
       </c>
     </row>
-    <row r="7" spans="1:16" s="18" customFormat="1" outlineLevel="1">
+    <row r="7" spans="1:16" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A7" s="25" t="s">
         <v>24</v>
       </c>
@@ -15858,7 +15858,7 @@
         <v>190000000</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="37" customFormat="1" outlineLevel="1">
+    <row r="8" spans="1:16" s="37" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A8" s="31"/>
       <c r="B8" s="32"/>
       <c r="C8" s="33"/>
@@ -15873,7 +15873,7 @@
       <c r="L8" s="34"/>
       <c r="M8" s="34"/>
     </row>
-    <row r="9" spans="1:16" s="18" customFormat="1">
+    <row r="9" spans="1:16" s="18" customFormat="1" ht="13.5">
       <c r="A9" s="29" t="s">
         <v>23</v>
       </c>
@@ -30619,21 +30619,21 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:P830"/>
-  <sheetFormatPr defaultColWidth="5.375" defaultRowHeight="13.5" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="5.3984375" defaultRowHeight="13.15" outlineLevelRow="2"/>
   <cols>
-    <col min="1" max="1" width="16.75" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.75" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.875" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.625" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.75" style="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="10.25" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.75" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.75" style="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.375" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="5.375" style="6"/>
+    <col min="1" max="1" width="16.73046875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.73046875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.86328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.46484375" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.3984375" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.46484375" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.59765625" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.73046875" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.73046875" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.73046875" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.3984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="5.3984375" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -30651,7 +30651,7 @@
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" ht="13.5">
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
@@ -30663,7 +30663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="18" customFormat="1" ht="27.75" thickBot="1">
+    <row r="3" spans="1:13" s="18" customFormat="1" ht="26.65" thickBot="1">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -30790,7 +30790,7 @@
         <v>162300000</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="18" customFormat="1" outlineLevel="1">
+    <row r="6" spans="1:13" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A6" s="25" t="s">
         <v>45</v>
       </c>
@@ -30945,7 +30945,7 @@
         <v>171000000</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="18" customFormat="1" outlineLevel="1">
+    <row r="10" spans="1:13" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A10" s="25" t="s">
         <v>28</v>
       </c>
@@ -31057,7 +31057,7 @@
         <v>32900000</v>
       </c>
     </row>
-    <row r="13" spans="1:13" s="18" customFormat="1" outlineLevel="1">
+    <row r="13" spans="1:13" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A13" s="25" t="s">
         <v>43</v>
       </c>
@@ -31169,7 +31169,7 @@
         <v>25200000</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="18" customFormat="1" outlineLevel="1">
+    <row r="16" spans="1:13" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A16" s="25" t="s">
         <v>39</v>
       </c>
@@ -31324,7 +31324,7 @@
         <v>220000000</v>
       </c>
     </row>
-    <row r="20" spans="1:16" s="18" customFormat="1" outlineLevel="1">
+    <row r="20" spans="1:16" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A20" s="25" t="s">
         <v>30</v>
       </c>
@@ -31436,7 +31436,7 @@
         <v>37000000</v>
       </c>
     </row>
-    <row r="23" spans="1:16" s="18" customFormat="1" outlineLevel="1">
+    <row r="23" spans="1:16" s="18" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A23" s="25" t="s">
         <v>24</v>
       </c>
@@ -31462,7 +31462,7 @@
         <v>227000000</v>
       </c>
     </row>
-    <row r="24" spans="1:16" s="37" customFormat="1" outlineLevel="1">
+    <row r="24" spans="1:16" s="37" customFormat="1" ht="13.5" outlineLevel="1">
       <c r="A24" s="31"/>
       <c r="B24" s="32"/>
       <c r="C24" s="33"/>
@@ -31477,7 +31477,7 @@
       <c r="L24" s="34"/>
       <c r="M24" s="34"/>
     </row>
-    <row r="25" spans="1:16" s="18" customFormat="1">
+    <row r="25" spans="1:16" s="18" customFormat="1" ht="13.5">
       <c r="A25" s="29" t="s">
         <v>23</v>
       </c>

</xml_diff>